<commit_message>
fix: apply explicit black font and solid white fill to excel files for 100% Android and dark mode compatibility
</commit_message>
<xml_diff>
--- a/assets/ejemplos excel alimentos/1_catalogo_base_alimentos.xlsx
+++ b/assets/ejemplos excel alimentos/1_catalogo_base_alimentos.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0,##0"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,8 +33,25 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -45,6 +62,24 @@
       <patternFill patternType="solid">
         <fgColor rgb="001E293B"/>
         <bgColor rgb="001E293B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E3A8A"/>
+        <bgColor rgb="001E3A8A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8FAFC"/>
+        <bgColor rgb="00F8FAFC"/>
       </patternFill>
     </fill>
   </fills>
@@ -74,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -85,6 +120,27 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -452,433 +508,433 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Código</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Producto</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>Presentación</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>Precio Actual ($)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>Stock</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>Categoría</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>ART-001</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>Aceite Cañuelas 1.5L</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>Caja x 6 u.</t>
         </is>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="D2" s="8" t="n">
         <v>14400</v>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>Almacén</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>ART-002</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="10" t="inlineStr">
         <is>
           <t>Harina Pureza 000 1kg</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="10" t="inlineStr">
         <is>
           <t>Fardo x 10 u.</t>
         </is>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D3" s="11" t="n">
         <v>12500</v>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F3" s="10" t="inlineStr">
         <is>
           <t>Almacén</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>ART-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>Arroz Lucchetti Largo Fino 1kg</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>Fardo x 10 u.</t>
         </is>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="8" t="n">
         <v>16000</v>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>Almacén</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>ART-004</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>Fideos Matarazzo Guiseros 500g</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="10" t="inlineStr">
         <is>
           <t>Caja x 15 u.</t>
         </is>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="11" t="n">
         <v>18000</v>
       </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
         <is>
           <t>Almacén</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>ART-005</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Azúcar Ledesma Clásica 1kg</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>Fardo x 10 u.</t>
         </is>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="8" t="n">
         <v>11000</v>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>Almacén</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>ART-006</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>Puré de Tomate De Cecco 520g</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>Caja x 12 u.</t>
         </is>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" s="11" t="n">
         <v>9800</v>
       </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
         <is>
           <t>Almacén</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>ART-007</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Queso Cremoso La Paulina</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>Horma x 4kg</t>
         </is>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="D8" s="8" t="n">
         <v>28000</v>
       </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
         <is>
           <t>Lácteos y Fríos</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>ART-008</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>Leche Entera La Serenísima 1L</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>Caja x 12 u.</t>
         </is>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="D9" s="11" t="n">
         <v>15600</v>
       </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
         <is>
           <t>Lácteos y Fríos</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>ART-009</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Yogur Firme Ilolay 120g</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>Pack x 8 u.</t>
         </is>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="D10" s="8" t="n">
         <v>6400</v>
       </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
         <is>
           <t>Lácteos y Fríos</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>ART-010</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Gaseosa Coca Cola 2.25L</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" s="10" t="inlineStr">
         <is>
           <t>Pack x 6 u.</t>
         </is>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="D11" s="11" t="n">
         <v>19200</v>
       </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
         <is>
           <t>Bebidas</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>ART-011</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Cerveza Quilmes Clásica 1L</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>Cajón x 12 u.</t>
         </is>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="D12" s="8" t="n">
         <v>24000</v>
       </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
         <is>
           <t>Bebidas</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>ART-012</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>Agua Mineral Villavicencio 2L</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C13" s="10" t="inlineStr">
         <is>
           <t>Pack x 6 u.</t>
         </is>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="D13" s="11" t="n">
         <v>8400</v>
       </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
         <is>
           <t>Bebidas</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>ART-013</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Yerba Playadito 1kg</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>Fardo x 10 u.</t>
         </is>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="D14" s="8" t="n">
         <v>38000</v>
       </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
         <is>
           <t>Almacén</t>
         </is>

</xml_diff>